<commit_message>
Ensure exact Batch Number extraction from packaging table, clean input placeholders, and leave batch empty if absent
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -608,6 +608,273 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>noon</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Household</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>INV000002</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-19 10:15:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>GENERAL PURPOSE</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Household</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>INV000003</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr"/>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-19 10:24:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Grease (Lithium-based) Extended Life</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Household</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>224</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>BIS 12203</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>INV000001</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Batch: BIS 12203</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-19 10:26:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>noon</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Household</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>INV000002</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-19 10:26:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>GENERAL PURPOSE</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Household</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>INV000003</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-19 10:26:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>